<commit_message>
处理空引用 txttableparser 中 debuginfo，改为 debug
</commit_message>
<xml_diff>
--- a/Assets/Data/Excel/BuildingData.xlsx
+++ b/Assets/Data/Excel/BuildingData.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="45">
   <si>
     <r>
       <rPr>
@@ -66,7 +66,7 @@
     <t xml:space="preserve">costs</t>
   </si>
   <si>
-    <t xml:space="preserve">maxLevel</t>
+    <t xml:space="preserve">levelIdl</t>
   </si>
   <si>
     <t xml:space="preserve">hitPoints</t>
@@ -184,7 +184,7 @@
     <t xml:space="preserve">(2, 2)</t>
   </si>
   <si>
-    <t xml:space="preserve">22=22|ss=33|s2=3</t>
+    <t xml:space="preserve">1|2</t>
   </si>
   <si>
     <t xml:space="preserve">Block</t>
@@ -202,16 +202,10 @@
     <t xml:space="preserve">sdaf</t>
   </si>
   <si>
-    <t xml:space="preserve">22=22|ss=33|s2=4</t>
-  </si>
-  <si>
     <t xml:space="preserve">NewInstance1</t>
   </si>
   <si>
     <t xml:space="preserve">s33</t>
-  </si>
-  <si>
-    <t xml:space="preserve">22=22|ss=33|s2=5</t>
   </si>
 </sst>
 </file>
@@ -604,11 +598,9 @@
         <v>60</v>
       </c>
       <c r="J4" s="3"/>
-      <c r="K4" s="2" t="s">
+      <c r="K4" s="2"/>
+      <c r="L4" s="3" t="s">
         <v>37</v>
-      </c>
-      <c r="L4" s="3" t="n">
-        <v>10</v>
       </c>
       <c r="M4" s="3"/>
       <c r="N4" s="3" t="n">
@@ -656,11 +648,9 @@
         <v>60</v>
       </c>
       <c r="J5" s="3"/>
-      <c r="K5" s="2" t="s">
-        <v>43</v>
-      </c>
+      <c r="K5" s="2"/>
       <c r="L5" s="3" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="M5" s="3"/>
       <c r="N5" s="3" t="n">
@@ -685,13 +675,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B6" s="3" t="n">
         <v>333</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
@@ -706,11 +696,9 @@
         <v>60</v>
       </c>
       <c r="J6" s="3"/>
-      <c r="K6" s="2" t="s">
-        <v>46</v>
-      </c>
+      <c r="K6" s="2"/>
       <c r="L6" s="3" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="M6" s="3"/>
       <c r="N6" s="3" t="n">

</xml_diff>